<commit_message>
Actualizar tabla de variables del ejercicio 2
Se agrega la tabla de variables del ejercicio 2: Verificación de combustible.
</commit_message>
<xml_diff>
--- a/ProyectoMision/Diagramas/Tabla_variables_mision.xlsx
+++ b/ProyectoMision/Diagramas/Tabla_variables_mision.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alexanderpenaranda/Library/Mobile Documents/com~apple~CloudDocs/DocUCenfotec/Segundo_cuatriestre/Principios de Programación 1/Viaje espacial proyct/ProyectoProgra1MisionOrbita/ProyectoMision/Diagramas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BFD9DB35-ACB2-2B4B-9514-3458BE9D2DD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B366946C-4CC5-1440-A460-E1BEAB26EAB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19880" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ejercicio 1 Pag A" sheetId="1" r:id="rId1"/>
     <sheet name="Ejercicio 1 Pag B" sheetId="10" r:id="rId2"/>
-    <sheet name="Ejercicio 2" sheetId="5" r:id="rId3"/>
-    <sheet name="Ejercicio 3" sheetId="8" r:id="rId4"/>
+    <sheet name="Ejercicio 2 Pag A" sheetId="5" r:id="rId3"/>
+    <sheet name="Ejercicio 3 Pag B " sheetId="8" r:id="rId4"/>
     <sheet name="Ejercicio 4" sheetId="9" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="97">
   <si>
     <t>Nombre</t>
   </si>
@@ -236,12 +236,6 @@
     <t>Tabla de Casos de prueba  Ejercicio 2: Verificación de combustible</t>
   </si>
   <si>
-    <t>cantidad_combustible_disponible</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cantidad de combustible desponible en la nave ingresado por  el usuraio </t>
-  </si>
-  <si>
     <t xml:space="preserve">Aceptado </t>
   </si>
   <si>
@@ -252,13 +246,82 @@
   </si>
   <si>
     <t>Nombre de la misión:  Horizonte/ Cantidad total de tripulantes: 4/ Duración estimada hasta el destino: 8/ Combustible requerido para llegar al destino: 64/ Combustible requerido para regresar de la misión: 64/ Reserva de combustible de la nave: 10/ Combustible total requerido para la misión: 138/ Reserva de oxígeno para la misión: 5/ Oxígeno total requerido para la misión: 133/ Reserva de energía para la misión: 10/ Energía total requerida para la misión: 90/ Reserva de provisiones para la misión: 3/ Provisiones totales para la misión: 67</t>
+  </si>
+  <si>
+    <t xml:space="preserve">combustible_disponible </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entrada </t>
+  </si>
+  <si>
+    <t>El usuario ingresa el combustible que requiere la nave para el regreso de la misión.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El usuario ingresa el combustible disponible de la nave. </t>
+  </si>
+  <si>
+    <t>Cantidad fija de combustible necesaria para la reserva de emergencia : 10.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Constante </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ILIMITE_ADVERTENCIA </t>
+  </si>
+  <si>
+    <t xml:space="preserve">int </t>
+  </si>
+  <si>
+    <t>Las 10 unidades con las que comparás el margen adicional para saber si es bajo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">combustible_adicional </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cantidad de combustible que sobra o falta después de restar el combustible total requerido al combustible disponible.uestra el combustible adicionla que tiene la nave </t>
+  </si>
+  <si>
+    <t>Combustible disponible</t>
+  </si>
+  <si>
+    <t>Combustible requerido para llegar</t>
+  </si>
+  <si>
+    <t>Combustible requerido para regresar</t>
+  </si>
+  <si>
+    <t> Reserva de emergencia</t>
+  </si>
+  <si>
+    <t>Combustible total requerido</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Salida </t>
+  </si>
+  <si>
+    <t>El programa muesta el combustible disponible de la nave para la misión.</t>
+  </si>
+  <si>
+    <t>El programa muesta el combustible requerido de la nave para llegar al lugara de la misión.</t>
+  </si>
+  <si>
+    <t>El programa muesta el combustible requerido de la nave para regresar de la  misión.</t>
+  </si>
+  <si>
+    <t>El programa muesta el combustible de reserva que tiene  la nave para  misión.</t>
+  </si>
+  <si>
+    <t>El programa muesta el combustible total requerido para verificarar el combustible de la misión.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El usuario ingresa el combustible que requiere la nave para el destino de la misión. </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -296,6 +359,12 @@
     <font>
       <sz val="12"/>
       <name val="Aptos"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Century Gothic"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="5">
@@ -447,7 +516,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -541,209 +610,23 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="83">
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Aptos"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Aptos"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Aptos"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Aptos"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Aptos"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Aptos"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="0"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="2" tint="-0.749992370372631"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="64">
     <dxf>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
@@ -1471,194 +1354,6 @@
       </border>
     </dxf>
     <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Aptos"/>
-        <scheme val="none"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Aptos"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Aptos"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Aptos"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Aptos"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Aptos"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="0"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="2" tint="-0.749992370372631"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <font>
         <strike val="0"/>
         <outline val="0"/>
@@ -1834,198 +1529,6 @@
       </border>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Aptos"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Aptos"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Aptos"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Aptos"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Aptos"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Aptos"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="0"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="2" tint="-0.749992370372631"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <font>
         <strike val="0"/>
         <outline val="0"/>
@@ -2199,6 +1702,198 @@
         <top/>
         <bottom/>
       </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Aptos"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Aptos"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Aptos"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Aptos"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Aptos"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Aptos"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="2" tint="-0.749992370372631"/>
+        </patternFill>
+      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2214,127 +1909,97 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{30212B1C-8E81-1A4E-9C7A-90B6D25B2E12}" name="Tabla1" displayName="Tabla1" ref="C3:F25" totalsRowShown="0" headerRowDxfId="82" dataDxfId="80" headerRowBorderDxfId="81" tableBorderDxfId="79" totalsRowBorderDxfId="78">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{30212B1C-8E81-1A4E-9C7A-90B6D25B2E12}" name="Tabla1" displayName="Tabla1" ref="C3:F25" totalsRowShown="0" headerRowDxfId="53" dataDxfId="51" headerRowBorderDxfId="52" tableBorderDxfId="50" totalsRowBorderDxfId="49">
   <autoFilter ref="C3:F25" xr:uid="{30212B1C-8E81-1A4E-9C7A-90B6D25B2E12}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{E5F6FF96-3D8D-9446-B048-7D218A920F00}" name="Nombre" dataDxfId="77"/>
-    <tableColumn id="2" xr3:uid="{610D3F09-92F6-5C4B-A622-70D9FBE04EF5}" name="Tipo de dato" dataDxfId="76"/>
-    <tableColumn id="3" xr3:uid="{F9E23D55-BAC1-0641-8EC2-FEB3294A2437}" name="Descripción" dataDxfId="75"/>
-    <tableColumn id="4" xr3:uid="{BD8D5D6F-1FF6-F348-A3E5-E76123FF519C}" name="Clasificación" dataDxfId="74"/>
+    <tableColumn id="1" xr3:uid="{E5F6FF96-3D8D-9446-B048-7D218A920F00}" name="Nombre" dataDxfId="48"/>
+    <tableColumn id="2" xr3:uid="{610D3F09-92F6-5C4B-A622-70D9FBE04EF5}" name="Tipo de dato" dataDxfId="47"/>
+    <tableColumn id="3" xr3:uid="{F9E23D55-BAC1-0641-8EC2-FEB3294A2437}" name="Descripción" dataDxfId="46"/>
+    <tableColumn id="4" xr3:uid="{BD8D5D6F-1FF6-F348-A3E5-E76123FF519C}" name="Clasificación" dataDxfId="45"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D83CCF3F-B3B2-8446-B29D-6493DF4F96CB}" name="Tabla33" displayName="Tabla33" ref="H28:N31" totalsRowShown="0" headerRowDxfId="73" dataDxfId="72" tableBorderDxfId="71">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{40CE88EF-2D6B-3745-8808-4FA86DEE4DFF}" name="Tabla335" displayName="Tabla335" ref="D3:J6" totalsRowShown="0" headerRowDxfId="63" dataDxfId="62" tableBorderDxfId="61">
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{F71BAD39-C717-FF4E-900C-9457931413FB}" name="ID" dataDxfId="70"/>
-    <tableColumn id="2" xr3:uid="{DF9CF1DB-66E2-404A-80F2-3329F71A6C64}" name="Ejecicio" dataDxfId="69"/>
-    <tableColumn id="3" xr3:uid="{83E73783-D78C-4A4E-B631-36E9FC91D5FA}" name="Escenario" dataDxfId="68"/>
-    <tableColumn id="4" xr3:uid="{4E082AF0-2064-8845-9A6C-112AFB22483C}" name="Datos de entrada " dataDxfId="67"/>
-    <tableColumn id="5" xr3:uid="{2CA5EC4A-CE00-0744-8474-561B0B442E9C}" name="Resultado esperado" dataDxfId="66"/>
-    <tableColumn id="6" xr3:uid="{44C71504-D5F3-944B-93CB-AE501C1356F0}" name="Resultado Obtenido" dataDxfId="65"/>
-    <tableColumn id="7" xr3:uid="{ECA37BE3-B8C3-024E-B627-9BD1F699612F}" name="Estado" dataDxfId="64"/>
+    <tableColumn id="1" xr3:uid="{A051D503-7AB9-4042-B5B5-152806ADC4CD}" name="ID" dataDxfId="60"/>
+    <tableColumn id="2" xr3:uid="{F194BB1E-D39E-604D-AA25-268D5E58BA4E}" name="Ejecicio" dataDxfId="59"/>
+    <tableColumn id="3" xr3:uid="{FE7C624D-DB28-7647-BCCD-C817B6961CF4}" name="Escenario" dataDxfId="58"/>
+    <tableColumn id="4" xr3:uid="{5E476D27-2BDA-2648-B18C-B0CC1AD31DAE}" name="Datos de entrada " dataDxfId="57"/>
+    <tableColumn id="5" xr3:uid="{2E3E846B-F4D3-5049-90D2-E171D4CB5568}" name="Resultado esperado" dataDxfId="56"/>
+    <tableColumn id="6" xr3:uid="{09B53DA5-8144-8241-905E-A108B7D3ED97}" name="Resultado Obtenido" dataDxfId="55"/>
+    <tableColumn id="7" xr3:uid="{45C70A02-A9D9-4E4A-829B-09467C31F39B}" name="Estado" dataDxfId="54"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{40CE88EF-2D6B-3745-8808-4FA86DEE4DFF}" name="Tabla335" displayName="Tabla335" ref="D3:J6" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8" tableBorderDxfId="7">
-  <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{A051D503-7AB9-4042-B5B5-152806ADC4CD}" name="ID" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{F194BB1E-D39E-604D-AA25-268D5E58BA4E}" name="Ejecicio" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{FE7C624D-DB28-7647-BCCD-C817B6961CF4}" name="Escenario" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{5E476D27-2BDA-2648-B18C-B0CC1AD31DAE}" name="Datos de entrada " dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{2E3E846B-F4D3-5049-90D2-E171D4CB5568}" name="Resultado esperado" dataDxfId="2"/>
-    <tableColumn id="6" xr3:uid="{09B53DA5-8144-8241-905E-A108B7D3ED97}" name="Resultado Obtenido" dataDxfId="1"/>
-    <tableColumn id="7" xr3:uid="{45C70A02-A9D9-4E4A-829B-09467C31F39B}" name="Estado" dataDxfId="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{0B2B3120-6F78-1D4E-8370-5E2D745FA7EA}" name="Tabla18" displayName="Tabla18" ref="C3:F15" totalsRowShown="0" headerRowDxfId="44" dataDxfId="42" headerRowBorderDxfId="43" tableBorderDxfId="41" totalsRowBorderDxfId="40">
+  <autoFilter ref="C3:F15" xr:uid="{30212B1C-8E81-1A4E-9C7A-90B6D25B2E12}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{78678C7E-E971-0241-8812-1583865DCB13}" name="Nombre" dataDxfId="39"/>
+    <tableColumn id="2" xr3:uid="{AEC8C799-F440-0544-9501-3F8465CB5C88}" name="Tipo de dato" dataDxfId="38"/>
+    <tableColumn id="3" xr3:uid="{499CAD85-4510-F246-ACC9-549F2D510D7E}" name="Descripción" dataDxfId="37"/>
+    <tableColumn id="4" xr3:uid="{140EC8BC-E9D7-0B42-ADAA-FBB8BB816A62}" name="Clasificación" dataDxfId="36"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{0B2B3120-6F78-1D4E-8370-5E2D745FA7EA}" name="Tabla18" displayName="Tabla18" ref="C3:F25" totalsRowShown="0" headerRowDxfId="63" dataDxfId="61" headerRowBorderDxfId="62" tableBorderDxfId="60" totalsRowBorderDxfId="59">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{A75C2DA5-BA72-2244-A859-338CEDD10905}" name="Tabla1810" displayName="Tabla1810" ref="C3:F25" totalsRowShown="0" headerRowDxfId="35" dataDxfId="33" headerRowBorderDxfId="34" tableBorderDxfId="32" totalsRowBorderDxfId="31">
   <autoFilter ref="C3:F25" xr:uid="{30212B1C-8E81-1A4E-9C7A-90B6D25B2E12}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{78678C7E-E971-0241-8812-1583865DCB13}" name="Nombre" dataDxfId="58"/>
-    <tableColumn id="2" xr3:uid="{AEC8C799-F440-0544-9501-3F8465CB5C88}" name="Tipo de dato" dataDxfId="57"/>
-    <tableColumn id="3" xr3:uid="{499CAD85-4510-F246-ACC9-549F2D510D7E}" name="Descripción" dataDxfId="56"/>
-    <tableColumn id="4" xr3:uid="{140EC8BC-E9D7-0B42-ADAA-FBB8BB816A62}" name="Clasificación" dataDxfId="55"/>
+    <tableColumn id="1" xr3:uid="{DD284781-4C43-FC4E-B48F-1A497B5CFF2B}" name="Nombre" dataDxfId="30"/>
+    <tableColumn id="2" xr3:uid="{9D8A820A-2F9F-C643-9482-53F2B26A4409}" name="Tipo de dato" dataDxfId="29"/>
+    <tableColumn id="3" xr3:uid="{C36A0A94-A358-B547-A65A-9F68F93800FD}" name="Descripción" dataDxfId="28"/>
+    <tableColumn id="4" xr3:uid="{ED16F595-9C8C-5C46-9818-440739011BA3}" name="Clasificación" dataDxfId="27"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{0BF418B8-A65A-7D42-9557-4FEDBB08C137}" name="Tabla339" displayName="Tabla339" ref="J3:P6" totalsRowShown="0" headerRowDxfId="54" tableBorderDxfId="53">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{FC7FBD0C-FC5E-9346-8035-6B8644FF13E2}" name="Tabla33911" displayName="Tabla33911" ref="J3:P6" totalsRowShown="0" headerRowDxfId="26" tableBorderDxfId="25">
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{6F922E1E-D796-4640-AB20-6E275D082EF3}" name="ID" dataDxfId="52"/>
-    <tableColumn id="2" xr3:uid="{CEFBEB9C-BEC7-4D40-B8E0-38E8804DB7FF}" name="Ejecicio" dataDxfId="51"/>
-    <tableColumn id="3" xr3:uid="{7DEE4D7E-B532-0C46-B117-F9E410D05024}" name="Escenario" dataDxfId="50"/>
-    <tableColumn id="4" xr3:uid="{C6F88B72-0D33-504E-95D3-F61122D121B4}" name="Datos de entrada " dataDxfId="49"/>
-    <tableColumn id="5" xr3:uid="{39D68DF8-83F5-6E4D-9790-34CBDA3B4C61}" name="Resultado esperado" dataDxfId="48"/>
-    <tableColumn id="6" xr3:uid="{63B6D1B8-1E6B-CC4C-9F41-0965DD5E4899}" name="Resultado Obtenido" dataDxfId="47"/>
-    <tableColumn id="7" xr3:uid="{EE9EF043-FF3F-D14B-9973-E8015C6102C8}" name="Estado" dataDxfId="46"/>
+    <tableColumn id="1" xr3:uid="{AE793D69-EC0F-1D48-8C75-D4A26F1FCEA4}" name="ID" dataDxfId="24"/>
+    <tableColumn id="2" xr3:uid="{19A087F7-AADE-1C4E-825C-780A7BC9922A}" name="Ejecicio" dataDxfId="23"/>
+    <tableColumn id="3" xr3:uid="{70FB600C-0911-A84A-9E47-F862D277B544}" name="Escenario" dataDxfId="22"/>
+    <tableColumn id="4" xr3:uid="{D0BC218A-C7A2-6B48-A78E-52C9E5873625}" name="Datos de entrada " dataDxfId="21"/>
+    <tableColumn id="5" xr3:uid="{76BF6D37-E7DB-774C-BC3A-1BC2C559B85C}" name="Resultado esperado" dataDxfId="20"/>
+    <tableColumn id="6" xr3:uid="{2EA55792-084B-8D4F-9A36-C1C8694D10F3}" name="Resultado Obtenido" dataDxfId="19"/>
+    <tableColumn id="7" xr3:uid="{D29CE18B-A1B3-A748-8847-A49DE00DDC9B}" name="Estado" dataDxfId="18"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{A75C2DA5-BA72-2244-A859-338CEDD10905}" name="Tabla1810" displayName="Tabla1810" ref="C3:F25" totalsRowShown="0" headerRowDxfId="45" dataDxfId="43" headerRowBorderDxfId="44" tableBorderDxfId="42" totalsRowBorderDxfId="41">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{94A24452-ACF5-7542-9332-147F90D79AC6}" name="Tabla181012" displayName="Tabla181012" ref="C3:F25" totalsRowShown="0" headerRowDxfId="17" dataDxfId="15" headerRowBorderDxfId="16" tableBorderDxfId="14" totalsRowBorderDxfId="13">
   <autoFilter ref="C3:F25" xr:uid="{30212B1C-8E81-1A4E-9C7A-90B6D25B2E12}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{DD284781-4C43-FC4E-B48F-1A497B5CFF2B}" name="Nombre" dataDxfId="40"/>
-    <tableColumn id="2" xr3:uid="{9D8A820A-2F9F-C643-9482-53F2B26A4409}" name="Tipo de dato" dataDxfId="39"/>
-    <tableColumn id="3" xr3:uid="{C36A0A94-A358-B547-A65A-9F68F93800FD}" name="Descripción" dataDxfId="38"/>
-    <tableColumn id="4" xr3:uid="{ED16F595-9C8C-5C46-9818-440739011BA3}" name="Clasificación" dataDxfId="37"/>
+    <tableColumn id="1" xr3:uid="{1ED9CEB0-8A7A-6849-A654-40DE236B8C1D}" name="Nombre" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{25E07B31-738C-9C48-809C-0301C8BEE3CD}" name="Tipo de dato" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{B9B65B26-271E-E844-A859-5F9AF003D5F8}" name="Descripción" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{CFCEB362-E9BC-524E-8EB3-4BAF854781AD}" name="Clasificación" dataDxfId="9"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{FC7FBD0C-FC5E-9346-8035-6B8644FF13E2}" name="Tabla33911" displayName="Tabla33911" ref="J3:P6" totalsRowShown="0" headerRowDxfId="36" tableBorderDxfId="35">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{F73F803D-DF48-E541-A025-F550C01C3CBB}" name="Tabla3391113" displayName="Tabla3391113" ref="J3:P6" totalsRowShown="0" headerRowDxfId="8" tableBorderDxfId="7">
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{AE793D69-EC0F-1D48-8C75-D4A26F1FCEA4}" name="ID" dataDxfId="34"/>
-    <tableColumn id="2" xr3:uid="{19A087F7-AADE-1C4E-825C-780A7BC9922A}" name="Ejecicio" dataDxfId="33"/>
-    <tableColumn id="3" xr3:uid="{70FB600C-0911-A84A-9E47-F862D277B544}" name="Escenario" dataDxfId="32"/>
-    <tableColumn id="4" xr3:uid="{D0BC218A-C7A2-6B48-A78E-52C9E5873625}" name="Datos de entrada " dataDxfId="31"/>
-    <tableColumn id="5" xr3:uid="{76BF6D37-E7DB-774C-BC3A-1BC2C559B85C}" name="Resultado esperado" dataDxfId="30"/>
-    <tableColumn id="6" xr3:uid="{2EA55792-084B-8D4F-9A36-C1C8694D10F3}" name="Resultado Obtenido" dataDxfId="29"/>
-    <tableColumn id="7" xr3:uid="{D29CE18B-A1B3-A748-8847-A49DE00DDC9B}" name="Estado" dataDxfId="28"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{94A24452-ACF5-7542-9332-147F90D79AC6}" name="Tabla181012" displayName="Tabla181012" ref="C3:F25" totalsRowShown="0" headerRowDxfId="27" dataDxfId="25" headerRowBorderDxfId="26" tableBorderDxfId="24" totalsRowBorderDxfId="23">
-  <autoFilter ref="C3:F25" xr:uid="{30212B1C-8E81-1A4E-9C7A-90B6D25B2E12}"/>
-  <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{1ED9CEB0-8A7A-6849-A654-40DE236B8C1D}" name="Nombre" dataDxfId="22"/>
-    <tableColumn id="2" xr3:uid="{25E07B31-738C-9C48-809C-0301C8BEE3CD}" name="Tipo de dato" dataDxfId="21"/>
-    <tableColumn id="3" xr3:uid="{B9B65B26-271E-E844-A859-5F9AF003D5F8}" name="Descripción" dataDxfId="20"/>
-    <tableColumn id="4" xr3:uid="{CFCEB362-E9BC-524E-8EB3-4BAF854781AD}" name="Clasificación" dataDxfId="19"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{F73F803D-DF48-E541-A025-F550C01C3CBB}" name="Tabla3391113" displayName="Tabla3391113" ref="J3:P6" totalsRowShown="0" headerRowDxfId="18" tableBorderDxfId="17">
-  <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{A3317615-56F3-154E-9F50-964653E1B30C}" name="ID" dataDxfId="16"/>
-    <tableColumn id="2" xr3:uid="{DB231E64-153E-E543-BE36-187ED4AE608F}" name="Ejecicio" dataDxfId="15"/>
-    <tableColumn id="3" xr3:uid="{40CCE944-0A7C-5846-ACAB-D6BFCD053331}" name="Escenario" dataDxfId="14"/>
-    <tableColumn id="4" xr3:uid="{819D0678-0879-5845-8815-AD43139FDFF3}" name="Datos de entrada " dataDxfId="13"/>
-    <tableColumn id="5" xr3:uid="{2202A9F0-28E8-184B-9CA6-C3BF3E5902AC}" name="Resultado esperado" dataDxfId="12"/>
-    <tableColumn id="6" xr3:uid="{360D40A9-4035-784E-B066-22E8A2202856}" name="Resultado Obtenido" dataDxfId="11"/>
-    <tableColumn id="7" xr3:uid="{CD70569B-E308-A646-B229-A2639850EC1E}" name="Estado" dataDxfId="10"/>
+    <tableColumn id="1" xr3:uid="{A3317615-56F3-154E-9F50-964653E1B30C}" name="ID" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{DB231E64-153E-E543-BE36-187ED4AE608F}" name="Ejecicio" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{40CCE944-0A7C-5846-ACAB-D6BFCD053331}" name="Escenario" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{819D0678-0879-5845-8815-AD43139FDFF3}" name="Datos de entrada " dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{2202A9F0-28E8-184B-9CA6-C3BF3E5902AC}" name="Resultado esperado" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{360D40A9-4035-784E-B066-22E8A2202856}" name="Resultado Obtenido" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{CD70569B-E308-A646-B229-A2639850EC1E}" name="Estado" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2535,7 +2200,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="C2:N31"/>
+  <dimension ref="C2:F31"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="30" customHeight="1"/>
   <cols>
     <col min="3" max="3" width="35.83203125" style="4" customWidth="1"/>
@@ -2553,12 +2218,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="3:6" ht="30" customHeight="1">
-      <c r="C2" s="35" t="s">
+      <c r="C2" s="36" t="s">
         <v>66</v>
       </c>
-      <c r="D2" s="35"/>
-      <c r="E2" s="35"/>
-      <c r="F2" s="35"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
     </row>
     <row r="3" spans="3:6" ht="30" customHeight="1">
       <c r="C3" s="2" t="s">
@@ -2756,7 +2421,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="3:14" ht="30" customHeight="1">
+    <row r="17" spans="3:6" ht="30" customHeight="1">
       <c r="C17" s="11" t="s">
         <v>4</v>
       </c>
@@ -2770,7 +2435,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="18" spans="3:14" ht="30" customHeight="1">
+    <row r="18" spans="3:6" ht="30" customHeight="1">
       <c r="C18" s="11" t="s">
         <v>11</v>
       </c>
@@ -2784,7 +2449,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="19" spans="3:14" ht="30" customHeight="1">
+    <row r="19" spans="3:6" ht="30" customHeight="1">
       <c r="C19" s="15" t="s">
         <v>16</v>
       </c>
@@ -2798,7 +2463,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="20" spans="3:14" ht="30" customHeight="1">
+    <row r="20" spans="3:6" ht="30" customHeight="1">
       <c r="C20" s="15" t="s">
         <v>19</v>
       </c>
@@ -2812,7 +2477,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="21" spans="3:14" ht="30" customHeight="1">
+    <row r="21" spans="3:6" ht="30" customHeight="1">
       <c r="C21" s="11" t="s">
         <v>21</v>
       </c>
@@ -2826,7 +2491,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="22" spans="3:14" ht="30" customHeight="1">
+    <row r="22" spans="3:6" ht="30" customHeight="1">
       <c r="C22" s="15" t="s">
         <v>62</v>
       </c>
@@ -2840,7 +2505,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="23" spans="3:14" ht="30" customHeight="1">
+    <row r="23" spans="3:6" ht="30" customHeight="1">
       <c r="C23" s="11" t="s">
         <v>47</v>
       </c>
@@ -2854,7 +2519,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="24" spans="3:14" ht="30" customHeight="1">
+    <row r="24" spans="3:6" ht="30" customHeight="1">
       <c r="C24" s="11" t="s">
         <v>45</v>
       </c>
@@ -2868,7 +2533,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="25" spans="3:14" ht="30" customHeight="1">
+    <row r="25" spans="3:6" ht="30" customHeight="1">
       <c r="C25" s="16" t="s">
         <v>46</v>
       </c>
@@ -2882,119 +2547,19 @@
         <v>36</v>
       </c>
     </row>
-    <row r="27" spans="3:14" ht="21">
-      <c r="H27" s="36" t="s">
-        <v>67</v>
-      </c>
-      <c r="I27" s="36"/>
-      <c r="J27" s="36"/>
-      <c r="K27" s="36"/>
-      <c r="L27" s="36"/>
-      <c r="M27" s="36"/>
-      <c r="N27" s="36"/>
-    </row>
-    <row r="28" spans="3:14" ht="30" customHeight="1">
-      <c r="H28" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="I28" s="31" t="s">
-        <v>49</v>
-      </c>
-      <c r="J28" s="31" t="s">
-        <v>50</v>
-      </c>
-      <c r="K28" s="31" t="s">
-        <v>51</v>
-      </c>
-      <c r="L28" s="31" t="s">
-        <v>52</v>
-      </c>
-      <c r="M28" s="31" t="s">
-        <v>53</v>
-      </c>
-      <c r="N28" s="31" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="29" spans="3:14" ht="202" customHeight="1">
-      <c r="H29" s="12" t="s">
-        <v>64</v>
-      </c>
-      <c r="I29" s="34" t="s">
-        <v>55</v>
-      </c>
-      <c r="J29" s="32" t="s">
-        <v>63</v>
-      </c>
-      <c r="K29" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="L29" s="33" t="s">
-        <v>73</v>
-      </c>
-      <c r="M29" s="33" t="s">
-        <v>73</v>
-      </c>
-      <c r="N29" s="30" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="30" spans="3:14" ht="274" customHeight="1">
-      <c r="H30" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="I30" s="13" t="s">
-        <v>55</v>
-      </c>
-      <c r="J30" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="K30" s="13" t="s">
-        <v>60</v>
-      </c>
-      <c r="L30" s="33" t="s">
-        <v>74</v>
-      </c>
-      <c r="M30" s="33" t="s">
-        <v>74</v>
-      </c>
-      <c r="N30" s="30" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="31" spans="3:14" ht="199" customHeight="1">
-      <c r="H31" s="17" t="s">
-        <v>65</v>
-      </c>
-      <c r="I31" s="18" t="s">
-        <v>55</v>
-      </c>
-      <c r="J31" s="18" t="s">
-        <v>58</v>
-      </c>
-      <c r="K31" s="18" t="s">
-        <v>61</v>
-      </c>
-      <c r="L31" s="33" t="s">
-        <v>75</v>
-      </c>
-      <c r="M31" s="33" t="s">
-        <v>75</v>
-      </c>
-      <c r="N31" s="30" t="s">
-        <v>72</v>
-      </c>
-    </row>
+    <row r="27" spans="3:6" ht="15"/>
+    <row r="28" spans="3:6" ht="15"/>
+    <row r="29" spans="3:6" ht="15"/>
+    <row r="30" spans="3:6" ht="15"/>
+    <row r="31" spans="3:6" ht="15"/>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="1">
     <mergeCell ref="C2:F2"/>
-    <mergeCell ref="H27:N27"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
-  <tableParts count="2">
+  <tableParts count="1">
     <tablePart r:id="rId1"/>
-    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
@@ -3021,15 +2586,15 @@
   </cols>
   <sheetData>
     <row r="2" spans="4:10" ht="30" customHeight="1">
-      <c r="D2" s="36" t="s">
+      <c r="D2" s="35" t="s">
         <v>67</v>
       </c>
-      <c r="E2" s="36"/>
-      <c r="F2" s="36"/>
-      <c r="G2" s="36"/>
-      <c r="H2" s="36"/>
-      <c r="I2" s="36"/>
-      <c r="J2" s="36"/>
+      <c r="E2" s="35"/>
+      <c r="F2" s="35"/>
+      <c r="G2" s="35"/>
+      <c r="H2" s="35"/>
+      <c r="I2" s="35"/>
+      <c r="J2" s="35"/>
     </row>
     <row r="3" spans="4:10" ht="16">
       <c r="D3" s="8" t="s">
@@ -3054,7 +2619,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="4" spans="4:10" ht="409.6">
+    <row r="4" spans="4:10" ht="136">
       <c r="D4" s="12" t="s">
         <v>64</v>
       </c>
@@ -3068,16 +2633,16 @@
         <v>59</v>
       </c>
       <c r="H4" s="33" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="I4" s="33" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="J4" s="30" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="5" spans="4:10" ht="409.6">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="5" spans="4:10" ht="170">
       <c r="D5" s="12" t="s">
         <v>56</v>
       </c>
@@ -3091,16 +2656,16 @@
         <v>60</v>
       </c>
       <c r="H5" s="33" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I5" s="33" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="J5" s="30" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="6" spans="4:10" ht="409.6">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="6" spans="4:10" ht="136">
       <c r="D6" s="17" t="s">
         <v>65</v>
       </c>
@@ -3114,13 +2679,13 @@
         <v>61</v>
       </c>
       <c r="H6" s="33" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I6" s="33" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J6" s="30" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="27" ht="15"/>
@@ -3156,24 +2721,15 @@
     <col min="16" max="16" width="6.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="3:16" ht="30" customHeight="1">
-      <c r="C2" s="35" t="s">
+    <row r="2" spans="3:6" ht="30" customHeight="1">
+      <c r="C2" s="36" t="s">
         <v>68</v>
       </c>
-      <c r="D2" s="35"/>
-      <c r="E2" s="35"/>
-      <c r="F2" s="35"/>
-      <c r="J2" s="36" t="s">
-        <v>69</v>
-      </c>
-      <c r="K2" s="36"/>
-      <c r="L2" s="36"/>
-      <c r="M2" s="36"/>
-      <c r="N2" s="36"/>
-      <c r="O2" s="36"/>
-      <c r="P2" s="36"/>
-    </row>
-    <row r="3" spans="3:16" ht="30" customHeight="1">
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
+    </row>
+    <row r="3" spans="3:6" ht="30" customHeight="1">
       <c r="C3" s="2" t="s">
         <v>0</v>
       </c>
@@ -3186,48 +2742,22 @@
       <c r="F3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J3" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="K3" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="L3" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="M3" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="N3" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="O3" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="P3" s="8" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="4" spans="3:16" ht="30" customHeight="1">
-      <c r="C4" t="s">
-        <v>70</v>
+    </row>
+    <row r="4" spans="3:6" ht="30" customHeight="1">
+      <c r="C4" s="4" t="s">
+        <v>74</v>
       </c>
       <c r="D4" s="12" t="s">
         <v>9</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="F4" s="14"/>
-      <c r="J4" s="20"/>
-      <c r="K4" s="21"/>
-      <c r="L4" s="22"/>
-      <c r="M4" s="25"/>
-      <c r="N4" s="25"/>
-      <c r="O4" s="24"/>
-      <c r="P4" s="9"/>
-    </row>
-    <row r="5" spans="3:16" ht="30" customHeight="1">
+        <v>77</v>
+      </c>
+      <c r="F4" s="14" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="5" spans="3:6" ht="30" customHeight="1">
       <c r="C5" s="11" t="s">
         <v>16</v>
       </c>
@@ -3235,18 +2765,13 @@
         <v>9</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="F5" s="14"/>
-      <c r="J5" s="20"/>
-      <c r="K5" s="23"/>
-      <c r="L5" s="25"/>
-      <c r="M5" s="25"/>
-      <c r="N5" s="25"/>
-      <c r="O5" s="24"/>
-      <c r="P5" s="9"/>
-    </row>
-    <row r="6" spans="3:16" ht="30" customHeight="1">
+        <v>96</v>
+      </c>
+      <c r="F5" s="14" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6" spans="3:6" ht="30" customHeight="1">
       <c r="C6" s="11" t="s">
         <v>19</v>
       </c>
@@ -3254,130 +2779,137 @@
         <v>9</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="F6" s="14"/>
-      <c r="J6" s="26"/>
-      <c r="K6" s="27"/>
-      <c r="L6" s="28"/>
-      <c r="M6" s="28"/>
-      <c r="N6" s="28"/>
-      <c r="O6" s="29"/>
-      <c r="P6" s="10"/>
-    </row>
-    <row r="7" spans="3:16" ht="30" customHeight="1">
-      <c r="C7" s="11"/>
-      <c r="D7" s="12"/>
-      <c r="E7" s="13"/>
-      <c r="F7" s="14"/>
-    </row>
-    <row r="8" spans="3:16" ht="30" customHeight="1">
-      <c r="C8" s="11"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="13"/>
-      <c r="F8" s="14"/>
-    </row>
-    <row r="9" spans="3:16" ht="30" customHeight="1">
-      <c r="C9" s="11"/>
-      <c r="D9" s="12"/>
-      <c r="E9" s="13"/>
-      <c r="F9" s="14"/>
-    </row>
-    <row r="10" spans="3:16" ht="30" customHeight="1">
-      <c r="C10" s="11"/>
-      <c r="D10" s="12"/>
-      <c r="E10" s="13"/>
-      <c r="F10" s="14"/>
-    </row>
-    <row r="11" spans="3:16" ht="30" customHeight="1">
-      <c r="C11" s="11"/>
-      <c r="D11" s="12"/>
-      <c r="E11" s="13"/>
-      <c r="F11" s="14"/>
-    </row>
-    <row r="12" spans="3:16" ht="30" customHeight="1">
-      <c r="C12" s="11"/>
-      <c r="D12" s="12"/>
-      <c r="E12" s="13"/>
-      <c r="F12" s="14"/>
-    </row>
-    <row r="13" spans="3:16" ht="30" customHeight="1">
-      <c r="C13" s="11"/>
-      <c r="D13" s="12"/>
-      <c r="E13" s="13"/>
-      <c r="F13" s="14"/>
-    </row>
-    <row r="14" spans="3:16" ht="30" customHeight="1">
-      <c r="C14" s="11"/>
-      <c r="D14" s="12"/>
-      <c r="E14" s="13"/>
-      <c r="F14" s="14"/>
-    </row>
-    <row r="15" spans="3:16" ht="30" customHeight="1">
-      <c r="C15" s="11"/>
-      <c r="D15" s="12"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="14"/>
-    </row>
-    <row r="16" spans="3:16" ht="30" customHeight="1">
-      <c r="C16" s="11"/>
-      <c r="D16" s="12"/>
-      <c r="E16" s="13"/>
-      <c r="F16" s="14"/>
-    </row>
-    <row r="17" spans="3:19" ht="30" customHeight="1">
-      <c r="C17" s="11"/>
-      <c r="D17" s="12"/>
-      <c r="E17" s="13"/>
-      <c r="F17" s="14"/>
-    </row>
-    <row r="18" spans="3:19" ht="30" customHeight="1">
-      <c r="C18" s="11"/>
-      <c r="D18" s="12"/>
-      <c r="E18" s="13"/>
-      <c r="F18" s="14"/>
-    </row>
-    <row r="19" spans="3:19" ht="30" customHeight="1">
-      <c r="C19" s="15"/>
-      <c r="D19" s="12"/>
-      <c r="E19" s="13"/>
-      <c r="F19" s="14"/>
-    </row>
-    <row r="20" spans="3:19" ht="30" customHeight="1">
-      <c r="C20" s="15"/>
-      <c r="D20" s="12"/>
-      <c r="E20" s="13"/>
-      <c r="F20" s="14"/>
-    </row>
-    <row r="21" spans="3:19" ht="30" customHeight="1">
-      <c r="C21" s="11"/>
-      <c r="D21" s="12"/>
-      <c r="E21" s="13"/>
-      <c r="F21" s="14"/>
-    </row>
-    <row r="22" spans="3:19" ht="30" customHeight="1">
-      <c r="C22" s="15"/>
-      <c r="D22" s="12"/>
-      <c r="E22" s="13"/>
-      <c r="F22" s="14"/>
-    </row>
-    <row r="23" spans="3:19" ht="30" customHeight="1">
-      <c r="C23" s="11"/>
-      <c r="D23" s="12"/>
-      <c r="E23" s="13"/>
-      <c r="F23" s="14"/>
-    </row>
-    <row r="24" spans="3:19" ht="30" customHeight="1">
-      <c r="C24" s="11"/>
-      <c r="D24" s="12"/>
-      <c r="E24" s="13"/>
-      <c r="F24" s="14"/>
-    </row>
-    <row r="25" spans="3:19" ht="30" customHeight="1">
-      <c r="C25" s="16"/>
-      <c r="D25" s="17"/>
-      <c r="E25" s="18"/>
-      <c r="F25" s="19"/>
+        <v>76</v>
+      </c>
+      <c r="F6" s="14" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="7" spans="3:6" ht="30" customHeight="1">
+      <c r="C7" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="E7" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="F7" s="14" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="8" spans="3:6" ht="30" customHeight="1">
+      <c r="C8" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="E8" s="37" t="s">
+        <v>82</v>
+      </c>
+      <c r="F8" s="14" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="9" spans="3:6" ht="30" customHeight="1">
+      <c r="C9" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="E9" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="F9" s="14" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="3:6" ht="30" customHeight="1">
+      <c r="C10" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="E10" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="F10" s="14" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="3:6" ht="30" customHeight="1">
+      <c r="C11" s="38" t="s">
+        <v>85</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="E11" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="F11" s="14" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="12" spans="3:6" ht="30" customHeight="1">
+      <c r="C12" s="38" t="s">
+        <v>86</v>
+      </c>
+      <c r="D12" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="E12" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="F12" s="14" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="13" spans="3:6" ht="30" customHeight="1">
+      <c r="C13" s="38" t="s">
+        <v>87</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="E13" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="F13" s="14" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="14" spans="3:6" ht="30" customHeight="1">
+      <c r="C14" s="38" t="s">
+        <v>88</v>
+      </c>
+      <c r="D14" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="E14" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="F14" s="14" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="15" spans="3:6" ht="30" customHeight="1">
+      <c r="C15" s="38" t="s">
+        <v>89</v>
+      </c>
+      <c r="D15" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="E15" s="13" t="s">
+        <v>95</v>
+      </c>
+      <c r="F15" s="14" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="32" spans="3:19" s="6" customFormat="1" ht="30" customHeight="1">
       <c r="C32" s="4"/>
@@ -3398,15 +2930,13 @@
       <c r="S32"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="1">
     <mergeCell ref="C2:F2"/>
-    <mergeCell ref="J2:P2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
-  <tableParts count="2">
+  <tableParts count="1">
     <tablePart r:id="rId1"/>
-    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
@@ -3429,21 +2959,21 @@
   </cols>
   <sheetData>
     <row r="2" spans="3:16" ht="30" customHeight="1">
-      <c r="C2" s="35" t="s">
+      <c r="C2" s="36" t="s">
         <v>68</v>
       </c>
-      <c r="D2" s="35"/>
-      <c r="E2" s="35"/>
-      <c r="F2" s="35"/>
-      <c r="J2" s="36" t="s">
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
+      <c r="J2" s="35" t="s">
         <v>69</v>
       </c>
-      <c r="K2" s="36"/>
-      <c r="L2" s="36"/>
-      <c r="M2" s="36"/>
-      <c r="N2" s="36"/>
-      <c r="O2" s="36"/>
-      <c r="P2" s="36"/>
+      <c r="K2" s="35"/>
+      <c r="L2" s="35"/>
+      <c r="M2" s="35"/>
+      <c r="N2" s="35"/>
+      <c r="O2" s="35"/>
+      <c r="P2" s="35"/>
     </row>
     <row r="3" spans="3:16" ht="30" customHeight="1">
       <c r="C3" s="2" t="s">
@@ -3683,21 +3213,21 @@
   </cols>
   <sheetData>
     <row r="2" spans="3:16" ht="30" customHeight="1">
-      <c r="C2" s="35" t="s">
+      <c r="C2" s="36" t="s">
         <v>68</v>
       </c>
-      <c r="D2" s="35"/>
-      <c r="E2" s="35"/>
-      <c r="F2" s="35"/>
-      <c r="J2" s="36" t="s">
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
+      <c r="J2" s="35" t="s">
         <v>69</v>
       </c>
-      <c r="K2" s="36"/>
-      <c r="L2" s="36"/>
-      <c r="M2" s="36"/>
-      <c r="N2" s="36"/>
-      <c r="O2" s="36"/>
-      <c r="P2" s="36"/>
+      <c r="K2" s="35"/>
+      <c r="L2" s="35"/>
+      <c r="M2" s="35"/>
+      <c r="N2" s="35"/>
+      <c r="O2" s="35"/>
+      <c r="P2" s="35"/>
     </row>
     <row r="3" spans="3:16" ht="30" customHeight="1">
       <c r="C3" s="2" t="s">

</xml_diff>